<commit_message>
Add test data bundle, config, and synced English test reports.
Include Recipe_data README, English SemiInspection_10_TestCases.xlsx,
App.config/setup_env/config.json paths, and updated HTML/JUnit reports
after TC06 fix and English testcase migration.
</commit_message>
<xml_diff>
--- a/Automation_testcase/Test_cases/SemiInspection_10_TestCases.xlsx
+++ b/Automation_testcase/Test_cases/SemiInspection_10_TestCases.xlsx
@@ -90,24 +90,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Import Recipe 至 Recipe_data</t>
+          <t>Import Recipe to Recipe_data</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SemiInspectionDesktop.exe 已啟動；Recipe_data 可寫入</t>
+          <t>SemiInspectionDesktop.exe running; Recipe_data writable</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1. 點 Toolbar0「Import Recipe」(Ctrl+I)
-2. 選 InspectionRecipe_Sample.json
-3. 確認 RawData 表格</t>
+          <t>1. Click Toolbar0 Import Recipe (Ctrl+I)
+2. Select InspectionRecipe_Sample.json
+3. Verify RawData table</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>JSON 複製到 Recipe_data；DataGrid 顯示參數；日誌含 Import Recipe</t>
+          <t>JSON copied to Recipe_data; DataGrid shows parameters; log contains Import Recipe</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -142,23 +142,23 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>File Tree 顯示 Recipe_data</t>
+          <t>File Tree shows Recipe_data</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>應用程式已啟動</t>
+          <t>Application has started</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1. 檢視左側 File Tree
-2. 確認根節點 Recipe_data</t>
+          <t>1. View left File Tree
+2. Confirm root node Recipe_data</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>視窗標題 Semi Inspection Desktop；樹可見；Sample JSON 存在</t>
+          <t>Window title Semi Inspection Desktop; tree visible; Sample JSON exists</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -193,23 +193,23 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>RawData 參數表</t>
+          <t>RawData parameter table</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Recipe_data 含 InspectionRecipe_Sample.json</t>
+          <t>Recipe_data contains InspectionRecipe_Sample.json</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1. 點 Toolbar1「RawData」(Ctrl+E)
-2. 確認 DataGrid</t>
+          <t>1. Click Toolbar1 RawData (Ctrl+E)
+2. Confirm DataGrid</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>顯示 Category/Parameter/Value/Unit；日誌含 RawData</t>
+          <t>Shows Category/Parameter/Value/Unit; log contains RawData</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -244,23 +244,23 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Defect Chart 曲線圖</t>
+          <t>Defect Chart curve</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>已載入含 DefectSummary 的 Recipe</t>
+          <t>Recipe with DefectSummary loaded</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1. 點 Toolbar1「Defect Chart」(Ctrl+D)
-2. 檢視圖表區</t>
+          <t>1. Click Toolbar1 Defect Chart (Ctrl+D)
+2. View chart area</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>日誌含 Defect Chart 已繪製 5 類；X=DefectType Y=DefectCount</t>
+          <t>Log contains Defect Chart plotted 5 types; X=DefectType Y=DefectCount</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -295,23 +295,23 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>檔案樹雙擊開啟 Recipe</t>
+          <t>Double-click Recipe in file tree</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Recipe_data 有 InspectionRecipe_Sample.json</t>
+          <t>Recipe_data has InspectionRecipe_Sample.json</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1. 在 File Tree 雙擊 .json
-2. 檢視 RawData</t>
+          <t>1. Double-click .json in File Tree
+2. View RawData</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DataGrid 顯示 Recipe 參數；日誌含 Recipe</t>
+          <t>DataGrid shows Recipe parameters; log contains Recipe</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -346,22 +346,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>About 對話框</t>
+          <t>About dialog</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>應用程式已啟動</t>
+          <t>Application has started</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1. 點 Toolbar0「About」</t>
+          <t>1. Click Toolbar0 About</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>顯示 About（含 Recipe_data 路徑與 Inspection 功能說明）</t>
+          <t>Shows About (Recipe_data path and Inspection feature description)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -396,23 +396,23 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>匯入非 JSON 檔</t>
+          <t>Import non-JSON file</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>應用程式已啟動；_invalid_sample.txt 存在</t>
+          <t>Application has started; _invalid_sample.txt exists</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1. 點 Import Recipe
-2. 選擇 _invalid_sample.txt</t>
+          <t>1. Click Import Recipe
+2. Select _invalid_sample.txt</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>警告「請選擇 .json Recipe 檔案」；不寫入 TC01_import_copy.json</t>
+          <t>Warning Please select .json Recipe file; does not write TC01_import_copy.json</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -447,23 +447,23 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>無 Recipe 時繪圖</t>
+          <t>Chart without Recipe</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>重新啟動後尚未載入 Recipe</t>
+          <t>Relaunched without loaded Recipe</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1. 直接點 Defect Chart
-2. 關閉提示（若有）</t>
+          <t>1. Click Defect Chart directly
+2. Close prompt if shown</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>提示無 DefectSummary 或自動載入失敗警告；不當機</t>
+          <t>Prompt for missing DefectSummary or auto-load warning; no crash</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -498,23 +498,23 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>開啟不存在 Recipe</t>
+          <t>Open non-existent Recipe</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>應用程式已啟動</t>
+          <t>Application has started</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1. Ctrl+E 開啟 RawData 檔案對話框
-2. 選 not_exist_99999.json</t>
+          <t>1. Ctrl+E open RawData file dialog
+2. Select not_exist_99999.json</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>顯示錯誤訊息；主視窗仍可操作</t>
+          <t>Shows error message; main window still operable</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -549,23 +549,23 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Run Inspection 模擬檢測</t>
+          <t>Run Inspection simulation</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>已載入 InspectionRecipe_Sample.json</t>
+          <t>InspectionRecipe_Sample.json loaded</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1. 點 Toolbar0「Run Inspection」(Ctrl+R)
-2. 檢視日誌</t>
+          <t>1. Click Toolbar0 Run Inspection (Ctrl+R)
+2. View log</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>日誌含 Run Inspection、Recipe 名稱、ToolID、DefectSummary 合計</t>
+          <t>Log contains Run Inspection, Recipe name, ToolID, DefectSummary total</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">

</xml_diff>